<commit_message>
Rework pipeline, AusTender collector, email template, and store
- AusTender collector rebuilt with pagination and $1M+ contract filter
- Pipeline extended with DB-backed dedup, URL suppression, and run.json output
- Email HTML template overhauled; Excel store gains new output methods
- Models updated with escalation and confidence fields
- Remove temp Excel lock file and stale brand asset

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kestrel_config.xlsx
+++ b/data/kestrel_config.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalation" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Writing_Style" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audience" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AusTender_Agencies" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,13 +32,67 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F364A"/>
+        <bgColor rgb="002F364A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+        <bgColor rgb="00DDEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4E1"/>
+        <bgColor rgb="00FFE4E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE7F6"/>
+        <bgColor rgb="00EDE7F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F7FA"/>
+        <bgColor rgb="00E0F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE9E7"/>
+        <bgColor rgb="00FBE9E7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,8 +107,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8855,4 +8920,926 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agency Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Department of Defence</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Primary ADF/military department</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Australian Defence Force</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ADF umbrella — matches ADF-prefixed agencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Australian Army</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Land force</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Royal Australian Navy</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Maritime force</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Royal Australian Air Force</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Air force</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Defence Housing Australia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Provides housing for ADF members</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Defence Science and Technology Group</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Also listed as DST Group or DSTG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Capability Acquisition and Sustainment</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>CASG — part of Defence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Joint Operations Command</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ADF joint command</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Australian Strategic Policy Institute</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Core Defence</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ASPI — defence think tank, may procure</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Australian Signals Directorate</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>ASD — cyber and signals intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Australian Security Intelligence</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>ASIO — domestic security</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Australian Secret Intelligence</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>ASIS — foreign intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Office of National Intelligence</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>ONI — coordinates intelligence community</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Defence Intelligence Organisation</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>DIO — strategic intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Australian Geospatial-Intelligence</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>AGO — mapping and geospatial intel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Australian Cyber Security Centre</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Intelligence</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>ACSC — part of ASD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Department of Home Affairs</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio includes Border Force and AFP policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Australian Border Force</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>ABF — border protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Australian Federal Police</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>AFP — national policing, counter-terrorism</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Australian Maritime Safety Authority</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>AMSA — maritime safety and security</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Emergency Management Australia</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>EMA — national emergency coordination</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>National Emergency Management Agency</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Border &amp; Security</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>NEMA — successor to EMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Australian Space Agency</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Space &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>National space policy and programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Australian Nuclear Science and Technology</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Space &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>ANSTO — nuclear technology, AUKUS relevance</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Australian Radiation Protection</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Space &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>ARPANSA — radiation and nuclear safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Defence Science and Technology</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Space &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Alternate naming for DST Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Department of Industry</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Industry &amp; Export</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>DISR — sovereign industry and resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Department of Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Industry &amp; Export</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>DFAT — defence diplomacy and export controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Export Finance Australia</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Industry &amp; Export</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>EFA — defence export financing</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Australian Trade and Investment</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Industry &amp; Export</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Austrade — includes defence exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Defence SA</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>State Agency</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>South Australia defence industry office</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Defence West</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>State Agency</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Western Australia defence industry office</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Defence NSW</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>State Agency</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>New South Wales defence industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Defence Queensland</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>State Agency</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Queensland defence industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Queensland Defence Science Alliance</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>State Agency</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>QDSA — QLD defence R&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Department of the Prime Minister</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>National Security</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>PM&amp;C — national security policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>National Security Committee</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>National Security</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>NSC secretariat procurements</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Attorney-General</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>National Security</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>AG — national security legislation</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Australian Criminal Intelligence</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>National Security</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>ACIC — criminal intelligence</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>